<commit_message>
Funktioniert, nur noch code refactoren und release build updaten
</commit_message>
<xml_diff>
--- a/FATI_WordGenerator/Resources/Input.xlsx
+++ b/FATI_WordGenerator/Resources/Input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\polise\source\repos\FATI_WordGenerator\FATI_WordGenerator\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38E51FF-6E6F-4851-AB63-DD669D3616FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A58AA47-52E4-4153-BEF0-2EC3D83A6436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6255" yWindow="4050" windowWidth="28800" windowHeight="15345" xr2:uid="{2E3EC6A4-35A1-495C-9A86-58B7DC168D52}"/>
+    <workbookView xWindow="17115" yWindow="6750" windowWidth="28800" windowHeight="15345" xr2:uid="{2E3EC6A4-35A1-495C-9A86-58B7DC168D52}"/>
   </bookViews>
   <sheets>
     <sheet name="Adresse" sheetId="1" r:id="rId1"/>
@@ -51,9 +51,6 @@
     <t>Ort</t>
   </si>
   <si>
-    <t>Mittelgasse</t>
-  </si>
-  <si>
     <t>Wien</t>
   </si>
   <si>
@@ -76,6 +73,9 @@
   </si>
   <si>
     <t>Regie HA</t>
+  </si>
+  <si>
+    <t>Erion</t>
   </si>
 </sst>
 </file>
@@ -478,9 +478,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28.5">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2">
         <v>8</v>
@@ -489,7 +489,7 @@
         <v>1060</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -504,16 +504,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="30">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -521,10 +521,10 @@
         <v>18</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="D2" s="2">
         <v>50</v>
@@ -535,10 +535,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2">
         <v>45</v>

</xml_diff>

<commit_message>
First draft after long time
</commit_message>
<xml_diff>
--- a/FATI_WordGenerator/Resources/Input.xlsx
+++ b/FATI_WordGenerator/Resources/Input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\polise\source\repos\FATI_WordGenerator\FATI_WordGenerator\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF3DA84-9FDE-4C43-BF23-B8C6A0D65107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49CBDC6-B53F-4C82-B7F9-D4DAC2F1D331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{2E3EC6A4-35A1-495C-9A86-58B7DC168D52}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2E3EC6A4-35A1-495C-9A86-58B7DC168D52}"/>
   </bookViews>
   <sheets>
     <sheet name="Adresse" sheetId="1" r:id="rId1"/>
@@ -45,9 +45,6 @@
     <t>Nr</t>
   </si>
   <si>
-    <t>Bezirk</t>
-  </si>
-  <si>
     <t>Ort</t>
   </si>
   <si>
@@ -76,6 +73,9 @@
   </si>
   <si>
     <t>Schwechat</t>
+  </si>
+  <si>
+    <t>PLZ</t>
   </si>
 </sst>
 </file>
@@ -472,15 +472,15 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="28.5">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -489,7 +489,7 @@
         <v>2320</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -504,16 +504,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="30">
       <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -521,10 +521,10 @@
         <v>18</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="D2" s="2">
         <v>50</v>
@@ -535,10 +535,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="2">
         <v>45</v>

</xml_diff>

<commit_message>
Done, ready for adjustments
</commit_message>
<xml_diff>
--- a/FATI_WordGenerator/Resources/Input.xlsx
+++ b/FATI_WordGenerator/Resources/Input.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\polise\source\repos\FATI_WordGenerator\FATI_WordGenerator\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49CBDC6-B53F-4C82-B7F9-D4DAC2F1D331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DDAF0F6-6E1C-47D8-B5AB-668602C809B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2E3EC6A4-35A1-495C-9A86-58B7DC168D52}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{2E3EC6A4-35A1-495C-9A86-58B7DC168D52}"/>
   </bookViews>
   <sheets>
     <sheet name="Adresse" sheetId="1" r:id="rId1"/>
     <sheet name="Positionen" sheetId="2" r:id="rId2"/>
+    <sheet name="Firma" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>Straße</t>
   </si>
@@ -76,6 +77,21 @@
   </si>
   <si>
     <t>PLZ</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>ALLITECH Allgemeine Isoliertechnik GmbH</t>
+  </si>
+  <si>
+    <t>Wien</t>
+  </si>
+  <si>
+    <t>Große Schiffgasse</t>
+  </si>
+  <si>
+    <t>ATU</t>
   </si>
 </sst>
 </file>
@@ -463,6 +479,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA6935B8-3097-4B41-8CDD-183D5F8D2F85}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="16.75" customWidth="1"/>
+    <col min="3" max="3" width="8.5" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15">
       <c r="A1" s="1" t="s">
@@ -501,6 +522,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BE4830F-69C5-4E65-8EBB-8EB12C0E215B}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="3" max="3" width="24.25" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30">
       <c r="A1" s="1" t="s">
@@ -549,6 +573,64 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C24892E-EAAE-4E2A-A10C-D0B2E199BE20}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="28.75" customWidth="1"/>
+    <col min="3" max="3" width="18.25" customWidth="1"/>
+    <col min="4" max="4" width="14.625" customWidth="1"/>
+    <col min="5" max="5" width="19.375" customWidth="1"/>
+    <col min="6" max="6" width="20.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1020</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2">
+        <v>15586603</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6ecfacbe-31ad-493b-8038-696ca31d2afe}" enabled="1" method="Privileged" siteId="{763b2760-45c5-46d3-883e-29705bba49b7}" contentBits="0" removed="0"/>

</xml_diff>